<commit_message>
battle status bar update
</commit_message>
<xml_diff>
--- a/Battle_Library.xlsx
+++ b/Battle_Library.xlsx
@@ -2108,7 +2108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2194,21 +2194,21 @@
           <t>8</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>hg 1</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Individual</t>
+          <t>Shared</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>bad ass</t>
-        </is>
-      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -2232,10 +2232,14 @@
           <t>8</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>hg 2</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Individual</t>
+          <t>Shared</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -2245,6 +2249,74 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>NPC</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>War Priest</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>War Priest</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NPC</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ganador Marksman</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Ganador Marksman</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>bad ass</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Stop tracking generated/local files; sync working tree edits
- Untrack __pycache__/*.pyc (already gitignored, leftover from initial commit)
- Untrack encounter_state.json and workspace.json: live session/machine-local
  state that OneDrive already syncs directly; git tracking just produced
  constant diff noise
- Commit pending engine/template/data edits and old-files reorg
</commit_message>
<xml_diff>
--- a/Battle_Library.xlsx
+++ b/Battle_Library.xlsx
@@ -11,9 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ganador Patrol" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ganador Strike Force" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="The Elemental Anchoring" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Veyrath and the Wisps" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="test battle 1" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="test battle 2" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="test battle 2" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Karthmere elemental showdown" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Karthmere elemental showdown 2" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -582,54 +582,44 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BTL-004</t>
+          <t>BTL-006</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Veyrath and the Wisps</t>
+          <t>test battle 2</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Veyrath and the Wisps</t>
+          <t>test battle 2</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Ready</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>boss,veyrath</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Boss fight: Veyrath with a summoned wisp pack.</t>
+          <t>Draft</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BTL-005</t>
+          <t>BTL-007</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>test battle 1</t>
+          <t>Karthmere elemental showdown</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>test battle 1</t>
+          <t>Karthmere elemental showdown</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -639,24 +629,24 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BTL-006</t>
+          <t>BTL-008</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>test battle 2</t>
+          <t>Karthmere elemental showdown v2</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>test battle 2</t>
+          <t>Karthmere elemental showdown 2</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -669,7 +659,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>
@@ -1775,56 +1765,87 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>NPC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Rex</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>1</v>
+          <t>Hobgoblin</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Hobgoblin</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>hg 1</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Individual</t>
+          <t>Shared</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>NPC</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Prag</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>1</v>
+          <t>Hobgoblin</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Hobgoblin</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>hg 2</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Individual</t>
+          <t>Shared</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>NPC</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Roquist</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>1</v>
+          <t>Ganador Marksman</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Ganador Marksman</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1835,40 +1856,64 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>NPC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Giggles</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
+          <t>Hobgoblin</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Hobgoblin</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>Individual</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>novice</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>NPC</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Shaddow</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>1</v>
+          <t>Hobgoblin</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Hobgoblin</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>Individual</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>normal</t>
         </is>
       </c>
     </row>
@@ -1880,25 +1925,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Veyrath</t>
+          <t>Hobgoblin</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Veyrath</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>1</v>
+          <t>Hobgoblin</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>Individual</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>boss</t>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>veterian</t>
         </is>
       </c>
     </row>
@@ -1910,28 +1957,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Flame Wisp</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>3</v>
+          <t>Hobgoblin</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Hobgoblin</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Wisp Pack</t>
+          <t>elite attack</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Grouped Attacks</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>10</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>summoned by Veyrath (no stat tab; HP override)</t>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>elite</t>
         </is>
       </c>
     </row>
@@ -1946,7 +1997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2019,12 +2070,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Air Anchor Caster</t>
+          <t>Korrum</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Air Anchor Caster</t>
+          <t>Korrum</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -2046,12 +2097,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>War Mage</t>
+          <t>Veyrath</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>War Mage</t>
+          <t>Veyrath</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -2073,27 +2124,197 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hobgoblin</t>
+          <t>Earth Elemental</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Hobgoblin</t>
+          <t>Earth Elemental</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>red booties</t>
+          <t>Earth Mob Left</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Grouped Attacks</t>
+          <t>Individual</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NPC</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Fire Elemental</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Fire Elemental</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Fire Mob Left</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NPC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Earth Elemental</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Earth Elemental</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Earth Mob Right</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>NPC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Fire Elemental</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Fire Elemental</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Fire Mob Right</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>NPC</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Ganador Marksman</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Ganador Marksman</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Ganador Left</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>veterian</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>NPC</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Ganador Marksman</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Ganador Marksman</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Ganador Right</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>veterian</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2181,27 +2402,23 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Hobgoblin</t>
+          <t>Korrum</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hobgoblin</t>
+          <t>Korrum</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>hg 1</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>Individual</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -2219,27 +2436,23 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hobgoblin</t>
+          <t>Veyrath</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Hobgoblin</t>
+          <t>Veyrath</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>hg 2</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Shared</t>
+          <t>Individual</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -2257,18 +2470,24 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>War Priest</t>
+          <t>Earth Elemental</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>War Priest</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>Earth Elemental</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Earth Mob</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>Individual</t>
@@ -2289,18 +2508,24 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Ganador Marksman</t>
+          <t>Fire Elemental</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Ganador Marksman</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="inlineStr"/>
+          <t>Fire Elemental</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Fire Mob</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>Individual</t>
@@ -2310,12 +2535,92 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>bad ass</t>
-        </is>
-      </c>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NPC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Ganador Marksman</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Ganador Marksman</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Ganador Archers</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>veterian</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>NPC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ganador Veteran</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Ganador Veteran</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Ganador Swords</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>elite</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
delete optoins for npc
</commit_message>
<xml_diff>
--- a/Battle_Library.xlsx
+++ b/Battle_Library.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Battle Index" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ganador Patrol" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ganador Strike Force" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="The Elemental Anchoring" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="test battle 2" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Karthmere elemental showdown" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Karthmere elemental showdown 2" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Battle Index" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Ganador Patrol" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Ganador Strike Force" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="The Elemental Anchoring" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="test battle 2" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Karthmere elemental showdown" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Karthmere elemental showdown 2" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -659,7 +659,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
     </row>
@@ -2480,7 +2480,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -2518,7 +2518,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">

</xml_diff>